<commit_message>
Finalise requirement rules and scope notes
</commit_message>
<xml_diff>
--- a/Cameron_M1_Requirements_RTM (3).xlsx
+++ b/Cameron_M1_Requirements_RTM (3).xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RTM" sheetId="1" r:id="Rd8d56583adce4b31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="2" r:id="R7edb6c19c689459b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RTM" sheetId="1" r:id="R5bce19147d1d47ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="2" r:id="R3d4e717ca2954bac"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1923,60 +1923,82 @@
         <x:v>AC-NFR-009-2: Repeating a check from the same starting state gives the same outcome; deliberately invalid behaviour is detected.</x:v>
       </x:c>
     </x:row>
-    <x:row r="31" ht="46" customHeight="1">
+    <x:row r="31" ht="58" customHeight="1">
       <x:c r="A31" s="8" t="str">
         <x:v>Lifecycle</x:v>
       </x:c>
       <x:c r="B31" s="8" t="str">
-        <x:v>Proposed sequence: New → Assigned → In Progress → Resolved → Closed, with rejection from New and a recorded reason. Open means New, Assigned or In Progress. Reopening is not included.</x:v>
+        <x:v>Requests follow New → Assigned → In Progress → Resolved → Closed. A New request may be rejected with a recorded reason. Open means New, Assigned or In Progress. Reopening is not included.</x:v>
       </x:c>
       <x:c r="C31" s="8"/>
       <x:c r="D31" s="8"/>
       <x:c r="E31" s="8"/>
     </x:row>
-    <x:row r="32" ht="46" customHeight="1">
+    <x:row r="32" ht="58" customHeight="1">
       <x:c r="A32" s="8" t="str">
         <x:v>Permissions and feedback</x:v>
       </x:c>
       <x:c r="B32" s="8" t="str">
-        <x:v>Requesters see their own records and public updates. Staff access follows role/category permissions. Management sees service reporting. Feedback is proposed within the application; internal notes remain private.</x:v>
+        <x:v>Requesters view their own requests and public updates. Staff access follows role/category permissions. Management accesses service reporting. Feedback is provided within the application; internal staff notes remain private. Email notifications are not included in the initial version.</x:v>
       </x:c>
       <x:c r="C32" s="8"/>
       <x:c r="D32" s="8"/>
       <x:c r="E32" s="8"/>
     </x:row>
-    <x:row r="33" ht="46" customHeight="1">
+    <x:row r="33" ht="58" customHeight="1">
       <x:c r="A33" s="8" t="str">
         <x:v>Priority and overdue rules</x:v>
       </x:c>
       <x:c r="B33" s="8" t="str">
-        <x:v>Proposed priorities are Low, Normal and High, with Normal as default. An open request is overdue when the current time is later than its staff-set due time. Automatic escalation remains deferred.</x:v>
+        <x:v>Priorities are Low, Normal and High, with Normal as default. Authorised staff can change priorities and set due dates. An open request is overdue when its due time has passed. Requests without a due date are clearly identified and are not counted as overdue. Automatic escalation remains deferred.</x:v>
       </x:c>
       <x:c r="C33" s="8"/>
       <x:c r="D33" s="8"/>
       <x:c r="E33" s="8"/>
     </x:row>
-    <x:row r="34" ht="46" customHeight="1">
+    <x:row r="34" ht="58" customHeight="1">
       <x:c r="A34" s="8" t="str">
-        <x:v>Items to confirm</x:v>
+        <x:v>Categories</x:v>
       </x:c>
       <x:c r="B34" s="8" t="str">
-        <x:v>The team must confirm the category list, lifecycle, permission rules, feedback channel and optional attachments before sign-off. Attachments remain conditional under SR-IN-01 and are not claimed as fully specified here.</x:v>
+        <x:v>The initial categories are Facility Faults, Damaged Equipment, Security Concerns, IT Support, Maintenance, Lost Property and Other. Each request must use one category from this list.</x:v>
       </x:c>
       <x:c r="C34" s="8"/>
       <x:c r="D34" s="8"/>
       <x:c r="E34" s="8"/>
     </x:row>
-    <x:row r="35" ht="46" customHeight="1">
+    <x:row r="35" ht="58" customHeight="1">
       <x:c r="A35" s="8" t="str">
         <x:v>Quality targets</x:v>
       </x:c>
       <x:c r="B35" s="8" t="str">
-        <x:v>The numerical performance, usability and recovery targets are proposed pilot targets, subject to team agreement and hosting feasibility. They are not measured results.</x:v>
+        <x:v>The numerical performance, usability and recovery targets in NFR-002, NFR-004 and NFR-007 are acceptance targets for the pilot. Hosting options will be assessed against them in M2. Target changes follow change control. Achievement will be demonstrated through testing in later milestones.</x:v>
       </x:c>
       <x:c r="C35" s="8"/>
       <x:c r="D35" s="8"/>
       <x:c r="E35" s="8"/>
+    </x:row>
+    <x:row r="36" ht="58" customHeight="1">
+      <x:c r="A36" s="8" t="str">
+        <x:v>Attachments</x:v>
+      </x:c>
+      <x:c r="B36" s="8" t="str">
+        <x:v>File and photo uploads are deferred to future scope to limit storage, security and implementation work. Initial submissions contain a category, description and location.</x:v>
+      </x:c>
+      <x:c r="C36" s="8"/>
+      <x:c r="D36" s="8"/>
+      <x:c r="E36" s="8"/>
+    </x:row>
+    <x:row r="37" ht="58" customHeight="1">
+      <x:c r="A37" s="8" t="str">
+        <x:v>Scope boundaries</x:v>
+      </x:c>
+      <x:c r="B37" s="8" t="str">
+        <x:v>External messaging integrations, payments, multi-tenant support and native apps are excluded from the initial version. Attachments, automated escalation, public APIs, AI categorisation and multilingual support remain future scope. Technology and architecture decisions will be addressed in M2.</x:v>
+      </x:c>
+      <x:c r="C37" s="8"/>
+      <x:c r="D37" s="8"/>
+      <x:c r="E37" s="8"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1985,6 +2007,8 @@
     <x:mergeCell ref="B33:E33"/>
     <x:mergeCell ref="B34:E34"/>
     <x:mergeCell ref="B35:E35"/>
+    <x:mergeCell ref="B36:E36"/>
+    <x:mergeCell ref="B37:E37"/>
   </x:mergeCells>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="C2:C28">

</xml_diff>